<commit_message>
New figures for data at a glance
</commit_message>
<xml_diff>
--- a/downloads/latest-waiting-list.xlsx
+++ b/downloads/latest-waiting-list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs.sharepoint.com/sites/X24_PAT-UECandAP/Shared Documents/UEC and AP/RTT/Monthly RTT Report/25_26/202510 Oct/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs.sharepoint.com/sites/X24_PAT-UECandAP/Shared Documents/UEC and AP/RTT/Monthly RTT Report/25_26/202511 Nov/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{3DAF2501-AF2A-431F-A0A7-AB4BE36DDE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40861469-E22D-498C-A9AE-A8B8ADC5547F}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{3DAF2501-AF2A-431F-A0A7-AB4BE36DDE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47A27414-C726-47FC-9079-B059AFC63892}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Time Series" sheetId="6" r:id="rId1"/>
@@ -667,7 +667,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>April 2007 to October 2025</t>
+      <t>April 2007 to November 2025</t>
     </r>
   </si>
 </sst>
@@ -687,7 +687,7 @@
     <numFmt numFmtId="171" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="172" formatCode="#,##0.00000000000000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1957,67 +1957,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AX253"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="2" style="45" customWidth="1"/>
-    <col min="2" max="2" width="9.77734375" style="45" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="45" customWidth="1"/>
-    <col min="4" max="5" width="10.44140625" style="45" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" style="45" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" style="45" customWidth="1"/>
+    <col min="4" max="5" width="10.453125" style="45" customWidth="1"/>
     <col min="6" max="6" width="10" style="45" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="45" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" style="45" customWidth="1"/>
     <col min="8" max="8" width="10" style="45" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" style="45" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" style="45" customWidth="1"/>
     <col min="10" max="10" width="10" style="45" customWidth="1"/>
-    <col min="11" max="11" width="14.77734375" style="45" customWidth="1"/>
+    <col min="11" max="11" width="14.81640625" style="45" customWidth="1"/>
     <col min="12" max="12" width="10" style="45" customWidth="1"/>
-    <col min="13" max="13" width="14.77734375" style="45" customWidth="1"/>
+    <col min="13" max="13" width="14.81640625" style="45" customWidth="1"/>
     <col min="14" max="14" width="10" style="45" customWidth="1"/>
-    <col min="15" max="15" width="14.6640625" style="45" customWidth="1"/>
+    <col min="15" max="15" width="14.6328125" style="45" customWidth="1"/>
     <col min="16" max="16" width="10" style="76" customWidth="1"/>
-    <col min="17" max="17" width="14.77734375" style="76" customWidth="1"/>
+    <col min="17" max="17" width="14.81640625" style="76" customWidth="1"/>
     <col min="18" max="18" width="10" style="76" customWidth="1"/>
-    <col min="19" max="19" width="14.77734375" style="76" customWidth="1"/>
+    <col min="19" max="19" width="14.81640625" style="76" customWidth="1"/>
     <col min="20" max="20" width="10" style="45" customWidth="1"/>
-    <col min="21" max="21" width="14.77734375" style="45" customWidth="1"/>
-    <col min="22" max="22" width="17.44140625" style="45" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.44140625" style="45" customWidth="1"/>
-    <col min="24" max="24" width="19.44140625" style="45" customWidth="1"/>
-    <col min="25" max="25" width="15.44140625" style="45" customWidth="1"/>
-    <col min="26" max="27" width="10.44140625" style="45" customWidth="1"/>
+    <col min="21" max="21" width="14.81640625" style="45" customWidth="1"/>
+    <col min="22" max="22" width="17.453125" style="45" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.453125" style="45" customWidth="1"/>
+    <col min="24" max="24" width="19.453125" style="45" customWidth="1"/>
+    <col min="25" max="25" width="15.453125" style="45" customWidth="1"/>
+    <col min="26" max="27" width="10.453125" style="45" customWidth="1"/>
     <col min="28" max="30" width="10" style="45" customWidth="1"/>
-    <col min="31" max="31" width="15.44140625" style="45" customWidth="1"/>
-    <col min="32" max="33" width="10.44140625" style="45" customWidth="1"/>
+    <col min="31" max="31" width="15.453125" style="45" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" style="45" customWidth="1"/>
     <col min="34" max="36" width="10" style="45" customWidth="1"/>
-    <col min="37" max="37" width="15.44140625" style="45" customWidth="1"/>
+    <col min="37" max="37" width="15.453125" style="45" customWidth="1"/>
     <col min="38" max="38" width="10" style="45" customWidth="1"/>
-    <col min="39" max="39" width="15.44140625" style="45" customWidth="1"/>
-    <col min="40" max="40" width="10.77734375" style="45" customWidth="1"/>
-    <col min="41" max="41" width="9.44140625" style="45" customWidth="1"/>
-    <col min="42" max="42" width="12.44140625" style="45" customWidth="1"/>
-    <col min="43" max="43" width="10.44140625" style="45" customWidth="1"/>
+    <col min="39" max="39" width="15.453125" style="45" customWidth="1"/>
+    <col min="40" max="40" width="10.81640625" style="45" customWidth="1"/>
+    <col min="41" max="41" width="9.453125" style="45" customWidth="1"/>
+    <col min="42" max="42" width="12.453125" style="45" customWidth="1"/>
+    <col min="43" max="43" width="10.453125" style="45" customWidth="1"/>
     <col min="44" max="44" width="9" style="45" customWidth="1"/>
-    <col min="45" max="45" width="9.77734375" style="45" customWidth="1"/>
-    <col min="46" max="46" width="10.77734375" style="45" customWidth="1"/>
-    <col min="47" max="47" width="9.21875" style="45"/>
-    <col min="48" max="48" width="16.77734375" style="45" bestFit="1" customWidth="1"/>
-    <col min="49" max="16384" width="9.21875" style="45"/>
+    <col min="45" max="45" width="9.81640625" style="45" customWidth="1"/>
+    <col min="46" max="46" width="10.81640625" style="45" customWidth="1"/>
+    <col min="47" max="47" width="9.1796875" style="45"/>
+    <col min="48" max="48" width="16.81640625" style="45" bestFit="1" customWidth="1"/>
+    <col min="49" max="16384" width="9.1796875" style="45"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:48" ht="10.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:48" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:48" ht="10.5" customHeight="1"/>
+    <row r="2" spans="2:48" ht="15.5">
       <c r="B2" s="77" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="2:48" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:48" ht="15.5">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:48" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:48" ht="15.5">
       <c r="B4" s="77" t="s">
         <v>75</v>
       </c>
@@ -2053,7 +2053,7 @@
       <c r="AH4" s="30"/>
       <c r="AI4" s="30"/>
     </row>
-    <row r="5" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:48" ht="13">
       <c r="B5" s="77" t="s">
         <v>1</v>
       </c>
@@ -2088,7 +2088,7 @@
       <c r="AH5" s="30"/>
       <c r="AI5" s="30"/>
     </row>
-    <row r="6" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:48" ht="13">
       <c r="B6" s="77" t="s">
         <v>57</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="AH6" s="30"/>
       <c r="AI6" s="30"/>
     </row>
-    <row r="7" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:48" ht="13">
       <c r="B7" s="77" t="s">
         <v>2</v>
       </c>
@@ -2159,7 +2159,7 @@
       <c r="AH7" s="30"/>
       <c r="AI7" s="30"/>
     </row>
-    <row r="8" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:48" ht="13">
       <c r="B8" s="77" t="s">
         <v>3</v>
       </c>
@@ -2195,7 +2195,7 @@
       <c r="AH8" s="30"/>
       <c r="AI8" s="30"/>
     </row>
-    <row r="9" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:48" ht="13">
       <c r="B9" s="77" t="s">
         <v>72</v>
       </c>
@@ -2233,14 +2233,14 @@
       <c r="AH9" s="30"/>
       <c r="AI9" s="30"/>
     </row>
-    <row r="10" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:48" ht="13">
       <c r="B10" s="27"/>
       <c r="AJ10" s="78"/>
       <c r="AK10" s="78"/>
       <c r="AL10" s="78"/>
       <c r="AM10" s="78"/>
     </row>
-    <row r="11" spans="2:48" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:48" ht="34.5" customHeight="1">
       <c r="B11" s="28" t="s">
         <v>4</v>
       </c>
@@ -2302,7 +2302,7 @@
       <c r="AR11" s="74"/>
       <c r="AS11" s="75"/>
     </row>
-    <row r="12" spans="2:48" ht="66" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:48" ht="65">
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
       <c r="D12" s="57" t="s">
@@ -2430,7 +2430,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:48">
       <c r="B13" s="173" t="s">
         <v>34</v>
       </c>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="AV13" s="84"/>
     </row>
-    <row r="14" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:48">
       <c r="B14" s="173"/>
       <c r="C14" s="85">
         <v>39203</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="AV14" s="84"/>
     </row>
-    <row r="15" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:48">
       <c r="B15" s="173"/>
       <c r="C15" s="85">
         <v>39234</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="AV15" s="84"/>
     </row>
-    <row r="16" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:48">
       <c r="B16" s="173"/>
       <c r="C16" s="85">
         <v>39264</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="AV16" s="84"/>
     </row>
-    <row r="17" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:48">
       <c r="B17" s="173"/>
       <c r="C17" s="85">
         <v>39295</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="AV17" s="84"/>
     </row>
-    <row r="18" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:48">
       <c r="B18" s="173"/>
       <c r="C18" s="85">
         <v>39326</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="AV18" s="84"/>
     </row>
-    <row r="19" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:48">
       <c r="B19" s="173"/>
       <c r="C19" s="85">
         <v>39356</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="AV19" s="84"/>
     </row>
-    <row r="20" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:48">
       <c r="B20" s="173"/>
       <c r="C20" s="85">
         <v>39387</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="AV20" s="84"/>
     </row>
-    <row r="21" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:48">
       <c r="B21" s="173"/>
       <c r="C21" s="85">
         <v>39417</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="AV21" s="84"/>
     </row>
-    <row r="22" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:48">
       <c r="B22" s="173"/>
       <c r="C22" s="85">
         <v>39448</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="AV22" s="84"/>
     </row>
-    <row r="23" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:48">
       <c r="B23" s="173"/>
       <c r="C23" s="85">
         <v>39479</v>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="AV23" s="84"/>
     </row>
-    <row r="24" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:48">
       <c r="B24" s="173"/>
       <c r="C24" s="90">
         <v>39508</v>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="AV24" s="84"/>
     </row>
-    <row r="25" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:48">
       <c r="B25" s="173" t="s">
         <v>37</v>
       </c>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="AV25" s="84"/>
     </row>
-    <row r="26" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:48">
       <c r="B26" s="173"/>
       <c r="C26" s="85">
         <v>39569</v>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="AV26" s="84"/>
     </row>
-    <row r="27" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:48">
       <c r="B27" s="173"/>
       <c r="C27" s="85">
         <v>39600</v>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="AV27" s="84"/>
     </row>
-    <row r="28" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:48">
       <c r="B28" s="173"/>
       <c r="C28" s="85">
         <v>39630</v>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="AV28" s="84"/>
     </row>
-    <row r="29" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:48">
       <c r="B29" s="173"/>
       <c r="C29" s="85">
         <v>39661</v>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="AV29" s="84"/>
     </row>
-    <row r="30" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:48">
       <c r="B30" s="173"/>
       <c r="C30" s="85">
         <v>39692</v>
@@ -4774,7 +4774,7 @@
       </c>
       <c r="AV30" s="84"/>
     </row>
-    <row r="31" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:48">
       <c r="B31" s="173"/>
       <c r="C31" s="85">
         <v>39722</v>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="AV31" s="84"/>
     </row>
-    <row r="32" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:48">
       <c r="B32" s="173"/>
       <c r="C32" s="85">
         <v>39753</v>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="AV32" s="84"/>
     </row>
-    <row r="33" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:48">
       <c r="B33" s="173"/>
       <c r="C33" s="85">
         <v>39783</v>
@@ -5164,7 +5164,7 @@
       </c>
       <c r="AV33" s="84"/>
     </row>
-    <row r="34" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:48">
       <c r="B34" s="173"/>
       <c r="C34" s="85">
         <v>39814</v>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="AV34" s="84"/>
     </row>
-    <row r="35" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:48">
       <c r="B35" s="173"/>
       <c r="C35" s="85">
         <v>39845</v>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="AV35" s="84"/>
     </row>
-    <row r="36" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:48">
       <c r="B36" s="173"/>
       <c r="C36" s="90">
         <v>39873</v>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="AV36" s="84"/>
     </row>
-    <row r="37" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:48">
       <c r="B37" s="173" t="s">
         <v>38</v>
       </c>
@@ -5686,7 +5686,7 @@
       </c>
       <c r="AV37" s="84"/>
     </row>
-    <row r="38" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:48">
       <c r="B38" s="173"/>
       <c r="C38" s="85">
         <v>39934</v>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="AV38" s="84"/>
     </row>
-    <row r="39" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:48">
       <c r="B39" s="173"/>
       <c r="C39" s="85">
         <v>39965</v>
@@ -5946,7 +5946,7 @@
       </c>
       <c r="AV39" s="84"/>
     </row>
-    <row r="40" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:48">
       <c r="B40" s="173"/>
       <c r="C40" s="85">
         <v>39995</v>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AV40" s="84"/>
     </row>
-    <row r="41" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:48">
       <c r="B41" s="173"/>
       <c r="C41" s="85">
         <v>40026</v>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="AV41" s="84"/>
     </row>
-    <row r="42" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:48">
       <c r="B42" s="173"/>
       <c r="C42" s="85">
         <v>40057</v>
@@ -6336,7 +6336,7 @@
       </c>
       <c r="AV42" s="84"/>
     </row>
-    <row r="43" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:48">
       <c r="B43" s="173"/>
       <c r="C43" s="85">
         <v>40087</v>
@@ -6466,7 +6466,7 @@
       </c>
       <c r="AV43" s="84"/>
     </row>
-    <row r="44" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:48">
       <c r="B44" s="173"/>
       <c r="C44" s="85">
         <v>40118</v>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="AV44" s="84"/>
     </row>
-    <row r="45" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:48">
       <c r="B45" s="173"/>
       <c r="C45" s="85">
         <v>40148</v>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="AV45" s="84"/>
     </row>
-    <row r="46" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:48">
       <c r="B46" s="173"/>
       <c r="C46" s="85">
         <v>40179</v>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="AV46" s="84"/>
     </row>
-    <row r="47" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:48">
       <c r="B47" s="173"/>
       <c r="C47" s="85">
         <v>40210</v>
@@ -6986,7 +6986,7 @@
       </c>
       <c r="AV47" s="84"/>
     </row>
-    <row r="48" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:48">
       <c r="B48" s="173"/>
       <c r="C48" s="90">
         <v>40238</v>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="AV48" s="84"/>
     </row>
-    <row r="49" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:48">
       <c r="A49" s="102"/>
       <c r="B49" s="177" t="s">
         <v>39</v>
@@ -7249,7 +7249,7 @@
       </c>
       <c r="AV49" s="84"/>
     </row>
-    <row r="50" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:48">
       <c r="A50" s="102"/>
       <c r="B50" s="177"/>
       <c r="C50" s="104">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="AV50" s="84"/>
     </row>
-    <row r="51" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:48">
       <c r="A51" s="102"/>
       <c r="B51" s="177"/>
       <c r="C51" s="104">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="AV51" s="84"/>
     </row>
-    <row r="52" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:48">
       <c r="A52" s="102"/>
       <c r="B52" s="177"/>
       <c r="C52" s="104">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="AV52" s="84"/>
     </row>
-    <row r="53" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:48">
       <c r="A53" s="102"/>
       <c r="B53" s="177"/>
       <c r="C53" s="104">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="AV53" s="84"/>
     </row>
-    <row r="54" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:48">
       <c r="A54" s="102"/>
       <c r="B54" s="177"/>
       <c r="C54" s="104">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="AV54" s="84"/>
     </row>
-    <row r="55" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:48">
       <c r="A55" s="102"/>
       <c r="B55" s="177"/>
       <c r="C55" s="104">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="AV55" s="84"/>
     </row>
-    <row r="56" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:48">
       <c r="A56" s="102"/>
       <c r="B56" s="177"/>
       <c r="C56" s="104">
@@ -8166,7 +8166,7 @@
       </c>
       <c r="AV56" s="84"/>
     </row>
-    <row r="57" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:48">
       <c r="A57" s="102"/>
       <c r="B57" s="177"/>
       <c r="C57" s="104">
@@ -8297,7 +8297,7 @@
       </c>
       <c r="AV57" s="84"/>
     </row>
-    <row r="58" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:48">
       <c r="A58" s="102"/>
       <c r="B58" s="177"/>
       <c r="C58" s="104">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="AV58" s="84"/>
     </row>
-    <row r="59" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:48">
       <c r="A59" s="102"/>
       <c r="B59" s="177"/>
       <c r="C59" s="104">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="AV59" s="84"/>
     </row>
-    <row r="60" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:48">
       <c r="A60" s="102"/>
       <c r="B60" s="177"/>
       <c r="C60" s="105">
@@ -8690,7 +8690,7 @@
       </c>
       <c r="AV60" s="84"/>
     </row>
-    <row r="61" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:48">
       <c r="A61" s="102"/>
       <c r="B61" s="173" t="s">
         <v>40</v>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="AV61" s="84"/>
     </row>
-    <row r="62" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:48">
       <c r="A62" s="102"/>
       <c r="B62" s="173"/>
       <c r="C62" s="104">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="AV62" s="84"/>
     </row>
-    <row r="63" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:48">
       <c r="B63" s="173"/>
       <c r="C63" s="85">
         <v>40695</v>
@@ -9084,7 +9084,7 @@
       </c>
       <c r="AV63" s="84"/>
     </row>
-    <row r="64" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:48">
       <c r="B64" s="173"/>
       <c r="C64" s="85">
         <v>40725</v>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="AV64" s="84"/>
     </row>
-    <row r="65" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:48">
       <c r="B65" s="173"/>
       <c r="C65" s="85">
         <v>40756</v>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="AV65" s="84"/>
     </row>
-    <row r="66" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:48">
       <c r="B66" s="173"/>
       <c r="C66" s="85">
         <v>40787</v>
@@ -9474,7 +9474,7 @@
       </c>
       <c r="AV66" s="84"/>
     </row>
-    <row r="67" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:48">
       <c r="B67" s="173"/>
       <c r="C67" s="85">
         <v>40817</v>
@@ -9604,7 +9604,7 @@
       </c>
       <c r="AV67" s="84"/>
     </row>
-    <row r="68" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:48">
       <c r="B68" s="173"/>
       <c r="C68" s="85">
         <v>40848</v>
@@ -9734,7 +9734,7 @@
       </c>
       <c r="AV68" s="84"/>
     </row>
-    <row r="69" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:48">
       <c r="B69" s="173"/>
       <c r="C69" s="85">
         <v>40878</v>
@@ -9864,7 +9864,7 @@
       </c>
       <c r="AV69" s="84"/>
     </row>
-    <row r="70" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:48">
       <c r="B70" s="173"/>
       <c r="C70" s="85">
         <v>40909</v>
@@ -9994,7 +9994,7 @@
       </c>
       <c r="AV70" s="84"/>
     </row>
-    <row r="71" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:48">
       <c r="B71" s="173"/>
       <c r="C71" s="85">
         <v>40940</v>
@@ -10124,7 +10124,7 @@
       </c>
       <c r="AV71" s="84"/>
     </row>
-    <row r="72" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:48">
       <c r="B72" s="173"/>
       <c r="C72" s="90">
         <v>40969</v>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="AV72" s="84"/>
     </row>
-    <row r="73" spans="2:48" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:48" ht="12.75" customHeight="1">
       <c r="B73" s="173" t="s">
         <v>41</v>
       </c>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="AV73" s="84"/>
     </row>
-    <row r="74" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:48">
       <c r="B74" s="173"/>
       <c r="C74" s="85">
         <v>41030</v>
@@ -10516,7 +10516,7 @@
       </c>
       <c r="AV74" s="84"/>
     </row>
-    <row r="75" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:48">
       <c r="B75" s="173"/>
       <c r="C75" s="85">
         <v>41061</v>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="AV75" s="84"/>
     </row>
-    <row r="76" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:48">
       <c r="B76" s="173"/>
       <c r="C76" s="85">
         <v>41091</v>
@@ -10776,7 +10776,7 @@
       </c>
       <c r="AV76" s="84"/>
     </row>
-    <row r="77" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:48">
       <c r="B77" s="173"/>
       <c r="C77" s="85">
         <v>41122</v>
@@ -10906,7 +10906,7 @@
       </c>
       <c r="AV77" s="84"/>
     </row>
-    <row r="78" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:48">
       <c r="B78" s="173"/>
       <c r="C78" s="85">
         <v>41153</v>
@@ -11036,7 +11036,7 @@
       </c>
       <c r="AV78" s="84"/>
     </row>
-    <row r="79" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:48">
       <c r="B79" s="173"/>
       <c r="C79" s="85">
         <v>41183</v>
@@ -11166,7 +11166,7 @@
       </c>
       <c r="AV79" s="84"/>
     </row>
-    <row r="80" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:48">
       <c r="B80" s="173"/>
       <c r="C80" s="85">
         <v>41214</v>
@@ -11296,7 +11296,7 @@
       </c>
       <c r="AV80" s="84"/>
     </row>
-    <row r="81" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:48">
       <c r="B81" s="173"/>
       <c r="C81" s="85">
         <v>41244</v>
@@ -11426,7 +11426,7 @@
       </c>
       <c r="AV81" s="84"/>
     </row>
-    <row r="82" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:48">
       <c r="B82" s="173"/>
       <c r="C82" s="85">
         <v>41275</v>
@@ -11556,7 +11556,7 @@
       </c>
       <c r="AV82" s="84"/>
     </row>
-    <row r="83" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:48">
       <c r="B83" s="173"/>
       <c r="C83" s="85">
         <v>41306</v>
@@ -11686,7 +11686,7 @@
       </c>
       <c r="AV83" s="84"/>
     </row>
-    <row r="84" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:48">
       <c r="B84" s="173"/>
       <c r="C84" s="90">
         <v>41334</v>
@@ -11816,7 +11816,7 @@
       </c>
       <c r="AV84" s="84"/>
     </row>
-    <row r="85" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:48">
       <c r="B85" s="173" t="s">
         <v>42</v>
       </c>
@@ -11948,7 +11948,7 @@
       </c>
       <c r="AV85" s="84"/>
     </row>
-    <row r="86" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:48">
       <c r="B86" s="173"/>
       <c r="C86" s="85">
         <v>41395</v>
@@ -12078,7 +12078,7 @@
       </c>
       <c r="AV86" s="84"/>
     </row>
-    <row r="87" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:48">
       <c r="B87" s="173"/>
       <c r="C87" s="85">
         <v>41426</v>
@@ -12208,7 +12208,7 @@
       </c>
       <c r="AV87" s="84"/>
     </row>
-    <row r="88" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:48">
       <c r="B88" s="173"/>
       <c r="C88" s="85">
         <v>41456</v>
@@ -12338,7 +12338,7 @@
       </c>
       <c r="AV88" s="84"/>
     </row>
-    <row r="89" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:48">
       <c r="B89" s="173"/>
       <c r="C89" s="85">
         <v>41487</v>
@@ -12468,7 +12468,7 @@
       </c>
       <c r="AV89" s="84"/>
     </row>
-    <row r="90" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:48">
       <c r="B90" s="173"/>
       <c r="C90" s="85">
         <v>41518</v>
@@ -12598,7 +12598,7 @@
       </c>
       <c r="AV90" s="84"/>
     </row>
-    <row r="91" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:48">
       <c r="B91" s="173"/>
       <c r="C91" s="85">
         <v>41548</v>
@@ -12728,7 +12728,7 @@
       </c>
       <c r="AV91" s="84"/>
     </row>
-    <row r="92" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:48">
       <c r="B92" s="173"/>
       <c r="C92" s="85">
         <v>41579</v>
@@ -12858,7 +12858,7 @@
       </c>
       <c r="AV92" s="84"/>
     </row>
-    <row r="93" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:48">
       <c r="B93" s="173"/>
       <c r="C93" s="85">
         <v>41609</v>
@@ -12988,7 +12988,7 @@
       </c>
       <c r="AV93" s="84"/>
     </row>
-    <row r="94" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:48">
       <c r="B94" s="173"/>
       <c r="C94" s="85">
         <v>41640</v>
@@ -13118,7 +13118,7 @@
       </c>
       <c r="AV94" s="84"/>
     </row>
-    <row r="95" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:48">
       <c r="B95" s="173"/>
       <c r="C95" s="85">
         <v>41671</v>
@@ -13248,7 +13248,7 @@
       </c>
       <c r="AV95" s="84"/>
     </row>
-    <row r="96" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:48">
       <c r="B96" s="173"/>
       <c r="C96" s="90">
         <v>41699</v>
@@ -13378,7 +13378,7 @@
       </c>
       <c r="AV96" s="84"/>
     </row>
-    <row r="97" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:48">
       <c r="B97" s="173" t="s">
         <v>43</v>
       </c>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="AV97" s="84"/>
     </row>
-    <row r="98" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:48">
       <c r="B98" s="173"/>
       <c r="C98" s="85">
         <v>41760</v>
@@ -13640,7 +13640,7 @@
       </c>
       <c r="AV98" s="84"/>
     </row>
-    <row r="99" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:48">
       <c r="B99" s="173"/>
       <c r="C99" s="85">
         <v>41791</v>
@@ -13770,7 +13770,7 @@
       </c>
       <c r="AV99" s="84"/>
     </row>
-    <row r="100" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:48">
       <c r="B100" s="173"/>
       <c r="C100" s="85">
         <v>41821</v>
@@ -13900,7 +13900,7 @@
       </c>
       <c r="AV100" s="84"/>
     </row>
-    <row r="101" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:48">
       <c r="B101" s="173"/>
       <c r="C101" s="85">
         <v>41852</v>
@@ -14030,7 +14030,7 @@
       </c>
       <c r="AV101" s="84"/>
     </row>
-    <row r="102" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:48">
       <c r="B102" s="173"/>
       <c r="C102" s="85">
         <v>41883</v>
@@ -14160,7 +14160,7 @@
       </c>
       <c r="AV102" s="84"/>
     </row>
-    <row r="103" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:48">
       <c r="B103" s="173"/>
       <c r="C103" s="85">
         <v>41913</v>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="AV103" s="84"/>
     </row>
-    <row r="104" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:48">
       <c r="B104" s="173"/>
       <c r="C104" s="85">
         <v>41944</v>
@@ -14420,7 +14420,7 @@
       </c>
       <c r="AV104" s="84"/>
     </row>
-    <row r="105" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:48">
       <c r="B105" s="173"/>
       <c r="C105" s="85">
         <v>41974</v>
@@ -14550,7 +14550,7 @@
       </c>
       <c r="AV105" s="84"/>
     </row>
-    <row r="106" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:48">
       <c r="B106" s="173"/>
       <c r="C106" s="85">
         <v>42005</v>
@@ -14680,7 +14680,7 @@
       </c>
       <c r="AV106" s="84"/>
     </row>
-    <row r="107" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:48">
       <c r="B107" s="173"/>
       <c r="C107" s="85">
         <v>42036</v>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="AV107" s="84"/>
     </row>
-    <row r="108" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:48">
       <c r="B108" s="173"/>
       <c r="C108" s="90">
         <v>42064</v>
@@ -14940,7 +14940,7 @@
       </c>
       <c r="AV108" s="84"/>
     </row>
-    <row r="109" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:48">
       <c r="B109" s="173" t="s">
         <v>44</v>
       </c>
@@ -15072,7 +15072,7 @@
       </c>
       <c r="AV109" s="84"/>
     </row>
-    <row r="110" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:48">
       <c r="B110" s="173"/>
       <c r="C110" s="85">
         <v>42125</v>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="AV110" s="84"/>
     </row>
-    <row r="111" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:48">
       <c r="B111" s="173"/>
       <c r="C111" s="85">
         <v>42156</v>
@@ -15333,7 +15333,7 @@
       <c r="AT111" s="78"/>
       <c r="AV111" s="84"/>
     </row>
-    <row r="112" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:48">
       <c r="B112" s="173"/>
       <c r="C112" s="85">
         <v>42186</v>
@@ -15463,7 +15463,7 @@
       </c>
       <c r="AV112" s="84"/>
     </row>
-    <row r="113" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:50">
       <c r="B113" s="173"/>
       <c r="C113" s="85">
         <v>42217</v>
@@ -15593,7 +15593,7 @@
       </c>
       <c r="AV113" s="84"/>
     </row>
-    <row r="114" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:50">
       <c r="B114" s="173"/>
       <c r="C114" s="85">
         <v>42248</v>
@@ -15723,7 +15723,7 @@
       </c>
       <c r="AV114" s="84"/>
     </row>
-    <row r="115" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:50">
       <c r="B115" s="173"/>
       <c r="C115" s="85">
         <v>42278</v>
@@ -15853,7 +15853,7 @@
       </c>
       <c r="AV115" s="84"/>
     </row>
-    <row r="116" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:50">
       <c r="B116" s="173"/>
       <c r="C116" s="85">
         <v>42309</v>
@@ -15983,7 +15983,7 @@
       </c>
       <c r="AV116" s="84"/>
     </row>
-    <row r="117" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:50">
       <c r="B117" s="173"/>
       <c r="C117" s="85">
         <v>42339</v>
@@ -16113,7 +16113,7 @@
       </c>
       <c r="AV117" s="84"/>
     </row>
-    <row r="118" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:50">
       <c r="B118" s="173"/>
       <c r="C118" s="85">
         <v>42370</v>
@@ -16243,7 +16243,7 @@
       </c>
       <c r="AV118" s="84"/>
     </row>
-    <row r="119" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:50">
       <c r="B119" s="173"/>
       <c r="C119" s="85">
         <v>42401</v>
@@ -16373,7 +16373,7 @@
       </c>
       <c r="AV119" s="84"/>
     </row>
-    <row r="120" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:50">
       <c r="B120" s="173"/>
       <c r="C120" s="90">
         <v>42430</v>
@@ -16503,7 +16503,7 @@
       </c>
       <c r="AV120" s="84"/>
     </row>
-    <row r="121" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:50">
       <c r="B121" s="173" t="s">
         <v>45</v>
       </c>
@@ -16635,7 +16635,7 @@
       </c>
       <c r="AV121" s="84"/>
     </row>
-    <row r="122" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:50">
       <c r="B122" s="173"/>
       <c r="C122" s="85">
         <v>42491</v>
@@ -16765,7 +16765,7 @@
       </c>
       <c r="AV122" s="84"/>
     </row>
-    <row r="123" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:50">
       <c r="B123" s="173"/>
       <c r="C123" s="85">
         <v>42522</v>
@@ -16896,7 +16896,7 @@
       <c r="AT123" s="78"/>
       <c r="AV123" s="84"/>
     </row>
-    <row r="124" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:50">
       <c r="B124" s="173"/>
       <c r="C124" s="85">
         <v>42552</v>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="AV124" s="84"/>
     </row>
-    <row r="125" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:50">
       <c r="B125" s="173"/>
       <c r="C125" s="85">
         <v>42583</v>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="AV125" s="84"/>
     </row>
-    <row r="126" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:50">
       <c r="B126" s="173"/>
       <c r="C126" s="85">
         <v>42614</v>
@@ -17289,7 +17289,7 @@
       <c r="AV126" s="84"/>
       <c r="AW126" s="130"/>
     </row>
-    <row r="127" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:50">
       <c r="B127" s="173"/>
       <c r="C127" s="85">
         <v>42644</v>
@@ -17423,7 +17423,7 @@
       <c r="AW127" s="130"/>
       <c r="AX127" s="130"/>
     </row>
-    <row r="128" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:50">
       <c r="B128" s="173"/>
       <c r="C128" s="85">
         <v>42675</v>
@@ -17557,7 +17557,7 @@
       <c r="AW128" s="130"/>
       <c r="AX128" s="130"/>
     </row>
-    <row r="129" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:50">
       <c r="B129" s="173"/>
       <c r="C129" s="85">
         <v>42705</v>
@@ -17691,7 +17691,7 @@
       <c r="AW129" s="130"/>
       <c r="AX129" s="130"/>
     </row>
-    <row r="130" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:50">
       <c r="B130" s="173"/>
       <c r="C130" s="85">
         <v>42736</v>
@@ -17825,7 +17825,7 @@
       <c r="AW130" s="130"/>
       <c r="AX130" s="130"/>
     </row>
-    <row r="131" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:50">
       <c r="B131" s="173"/>
       <c r="C131" s="85">
         <v>42767</v>
@@ -17959,7 +17959,7 @@
       <c r="AW131" s="130"/>
       <c r="AX131" s="130"/>
     </row>
-    <row r="132" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:50">
       <c r="B132" s="173"/>
       <c r="C132" s="90">
         <v>42795</v>
@@ -18093,7 +18093,7 @@
       <c r="AW132" s="130"/>
       <c r="AX132" s="130"/>
     </row>
-    <row r="133" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:50">
       <c r="B133" s="173" t="s">
         <v>46</v>
       </c>
@@ -18229,7 +18229,7 @@
       <c r="AW133" s="130"/>
       <c r="AX133" s="130"/>
     </row>
-    <row r="134" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:50">
       <c r="B134" s="173"/>
       <c r="C134" s="85">
         <v>42856</v>
@@ -18363,7 +18363,7 @@
       <c r="AW134" s="130"/>
       <c r="AX134" s="130"/>
     </row>
-    <row r="135" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:50">
       <c r="B135" s="173"/>
       <c r="C135" s="85">
         <v>42887</v>
@@ -18497,7 +18497,7 @@
       <c r="AW135" s="130"/>
       <c r="AX135" s="130"/>
     </row>
-    <row r="136" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:50">
       <c r="B136" s="173"/>
       <c r="C136" s="85">
         <v>42917</v>
@@ -18630,7 +18630,7 @@
       <c r="AV136" s="84"/>
       <c r="AW136" s="130"/>
     </row>
-    <row r="137" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:50">
       <c r="B137" s="173"/>
       <c r="C137" s="85">
         <v>42948</v>
@@ -18763,7 +18763,7 @@
       <c r="AV137" s="84"/>
       <c r="AW137" s="130"/>
     </row>
-    <row r="138" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:50">
       <c r="B138" s="173"/>
       <c r="C138" s="85">
         <v>42979</v>
@@ -18893,7 +18893,7 @@
       </c>
       <c r="AV138" s="84"/>
     </row>
-    <row r="139" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:50">
       <c r="B139" s="173"/>
       <c r="C139" s="85">
         <v>43009</v>
@@ -19023,7 +19023,7 @@
       </c>
       <c r="AV139" s="84"/>
     </row>
-    <row r="140" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:50">
       <c r="B140" s="173"/>
       <c r="C140" s="85">
         <v>43040</v>
@@ -19153,7 +19153,7 @@
       </c>
       <c r="AV140" s="84"/>
     </row>
-    <row r="141" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:50">
       <c r="B141" s="173"/>
       <c r="C141" s="85">
         <v>43070</v>
@@ -19283,7 +19283,7 @@
       </c>
       <c r="AV141" s="84"/>
     </row>
-    <row r="142" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:50">
       <c r="B142" s="173"/>
       <c r="C142" s="85">
         <v>43101</v>
@@ -19413,7 +19413,7 @@
       </c>
       <c r="AV142" s="84"/>
     </row>
-    <row r="143" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:50">
       <c r="B143" s="173"/>
       <c r="C143" s="85">
         <v>43132</v>
@@ -19543,7 +19543,7 @@
       </c>
       <c r="AV143" s="84"/>
     </row>
-    <row r="144" spans="2:50" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:50">
       <c r="B144" s="173"/>
       <c r="C144" s="90">
         <v>43160</v>
@@ -19673,7 +19673,7 @@
       </c>
       <c r="AV144" s="84"/>
     </row>
-    <row r="145" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:48">
       <c r="B145" s="173" t="s">
         <v>47</v>
       </c>
@@ -19805,7 +19805,7 @@
       </c>
       <c r="AV145" s="84"/>
     </row>
-    <row r="146" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:48">
       <c r="B146" s="173"/>
       <c r="C146" s="85">
         <v>43221</v>
@@ -19935,7 +19935,7 @@
       </c>
       <c r="AV146" s="84"/>
     </row>
-    <row r="147" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:48">
       <c r="B147" s="173"/>
       <c r="C147" s="85">
         <v>43252</v>
@@ -20065,7 +20065,7 @@
       </c>
       <c r="AV147" s="84"/>
     </row>
-    <row r="148" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:48">
       <c r="B148" s="173"/>
       <c r="C148" s="85">
         <v>43282</v>
@@ -20195,7 +20195,7 @@
       </c>
       <c r="AV148" s="84"/>
     </row>
-    <row r="149" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:48">
       <c r="B149" s="173"/>
       <c r="C149" s="85">
         <v>43313</v>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="AV149" s="84"/>
     </row>
-    <row r="150" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:48">
       <c r="B150" s="173"/>
       <c r="C150" s="85">
         <v>43344</v>
@@ -20455,7 +20455,7 @@
       </c>
       <c r="AV150" s="84"/>
     </row>
-    <row r="151" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:48">
       <c r="B151" s="173"/>
       <c r="C151" s="85">
         <v>43374</v>
@@ -20585,7 +20585,7 @@
       </c>
       <c r="AV151" s="84"/>
     </row>
-    <row r="152" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:48">
       <c r="B152" s="173"/>
       <c r="C152" s="85">
         <v>43405</v>
@@ -20715,7 +20715,7 @@
       </c>
       <c r="AV152" s="84"/>
     </row>
-    <row r="153" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:48">
       <c r="B153" s="173"/>
       <c r="C153" s="85">
         <v>43435</v>
@@ -20845,7 +20845,7 @@
       </c>
       <c r="AV153" s="84"/>
     </row>
-    <row r="154" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:48">
       <c r="B154" s="173"/>
       <c r="C154" s="85">
         <v>43466</v>
@@ -20975,7 +20975,7 @@
       </c>
       <c r="AV154" s="84"/>
     </row>
-    <row r="155" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:48">
       <c r="B155" s="173"/>
       <c r="C155" s="85">
         <v>43497</v>
@@ -21105,7 +21105,7 @@
       </c>
       <c r="AV155" s="84"/>
     </row>
-    <row r="156" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:48">
       <c r="B156" s="173"/>
       <c r="C156" s="90">
         <v>43525</v>
@@ -21235,7 +21235,7 @@
       </c>
       <c r="AV156" s="84"/>
     </row>
-    <row r="157" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:48">
       <c r="B157" s="173" t="s">
         <v>48</v>
       </c>
@@ -21367,7 +21367,7 @@
       </c>
       <c r="AV157" s="84"/>
     </row>
-    <row r="158" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:48">
       <c r="B158" s="173"/>
       <c r="C158" s="85">
         <v>43586</v>
@@ -21497,7 +21497,7 @@
       </c>
       <c r="AV158" s="84"/>
     </row>
-    <row r="159" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:48">
       <c r="B159" s="173"/>
       <c r="C159" s="85">
         <v>43617</v>
@@ -21627,7 +21627,7 @@
       </c>
       <c r="AV159" s="84"/>
     </row>
-    <row r="160" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:48">
       <c r="B160" s="173"/>
       <c r="C160" s="85">
         <v>43647</v>
@@ -21757,7 +21757,7 @@
       </c>
       <c r="AV160" s="84"/>
     </row>
-    <row r="161" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:48">
       <c r="B161" s="173"/>
       <c r="C161" s="85">
         <v>43678</v>
@@ -21887,7 +21887,7 @@
       </c>
       <c r="AV161" s="84"/>
     </row>
-    <row r="162" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:48">
       <c r="B162" s="173"/>
       <c r="C162" s="85">
         <v>43709</v>
@@ -22017,7 +22017,7 @@
       </c>
       <c r="AV162" s="84"/>
     </row>
-    <row r="163" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:48">
       <c r="B163" s="173"/>
       <c r="C163" s="104">
         <v>43739</v>
@@ -22147,7 +22147,7 @@
       </c>
       <c r="AV163" s="84"/>
     </row>
-    <row r="164" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:48">
       <c r="B164" s="173"/>
       <c r="C164" s="104">
         <v>43770</v>
@@ -22277,7 +22277,7 @@
       </c>
       <c r="AV164" s="84"/>
     </row>
-    <row r="165" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:48">
       <c r="B165" s="173"/>
       <c r="C165" s="104">
         <v>43800</v>
@@ -22407,7 +22407,7 @@
       </c>
       <c r="AV165" s="84"/>
     </row>
-    <row r="166" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:48">
       <c r="B166" s="173"/>
       <c r="C166" s="104">
         <v>43831</v>
@@ -22537,7 +22537,7 @@
       </c>
       <c r="AV166" s="84"/>
     </row>
-    <row r="167" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:48">
       <c r="B167" s="173"/>
       <c r="C167" s="104">
         <v>43862</v>
@@ -22667,7 +22667,7 @@
       </c>
       <c r="AV167" s="84"/>
     </row>
-    <row r="168" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:48">
       <c r="B168" s="173"/>
       <c r="C168" s="105">
         <v>43891</v>
@@ -22797,7 +22797,7 @@
       </c>
       <c r="AV168" s="84"/>
     </row>
-    <row r="169" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:48">
       <c r="B169" s="173" t="s">
         <v>49</v>
       </c>
@@ -22929,7 +22929,7 @@
       </c>
       <c r="AV169" s="84"/>
     </row>
-    <row r="170" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:48">
       <c r="B170" s="173"/>
       <c r="C170" s="104">
         <v>43952</v>
@@ -23059,7 +23059,7 @@
       </c>
       <c r="AV170" s="84"/>
     </row>
-    <row r="171" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:48">
       <c r="B171" s="173"/>
       <c r="C171" s="104">
         <v>43983</v>
@@ -23189,7 +23189,7 @@
       </c>
       <c r="AV171" s="84"/>
     </row>
-    <row r="172" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:48">
       <c r="B172" s="173"/>
       <c r="C172" s="104">
         <v>44013</v>
@@ -23319,7 +23319,7 @@
       </c>
       <c r="AV172" s="84"/>
     </row>
-    <row r="173" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:48">
       <c r="B173" s="173"/>
       <c r="C173" s="104">
         <v>44044</v>
@@ -23449,7 +23449,7 @@
       </c>
       <c r="AV173" s="84"/>
     </row>
-    <row r="174" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:48">
       <c r="B174" s="173"/>
       <c r="C174" s="104">
         <v>44075</v>
@@ -23579,7 +23579,7 @@
       </c>
       <c r="AV174" s="84"/>
     </row>
-    <row r="175" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:48">
       <c r="B175" s="173"/>
       <c r="C175" s="104">
         <v>44105</v>
@@ -23709,7 +23709,7 @@
       </c>
       <c r="AV175" s="84"/>
     </row>
-    <row r="176" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:48">
       <c r="B176" s="173"/>
       <c r="C176" s="104">
         <v>44136</v>
@@ -23839,7 +23839,7 @@
       </c>
       <c r="AV176" s="84"/>
     </row>
-    <row r="177" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:48">
       <c r="B177" s="173"/>
       <c r="C177" s="104">
         <v>44166</v>
@@ -23969,7 +23969,7 @@
       </c>
       <c r="AV177" s="84"/>
     </row>
-    <row r="178" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:48">
       <c r="B178" s="173"/>
       <c r="C178" s="104">
         <v>44197</v>
@@ -24099,7 +24099,7 @@
       </c>
       <c r="AV178" s="84"/>
     </row>
-    <row r="179" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:48">
       <c r="B179" s="173"/>
       <c r="C179" s="104">
         <v>44228</v>
@@ -24229,7 +24229,7 @@
       </c>
       <c r="AV179" s="84"/>
     </row>
-    <row r="180" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:48">
       <c r="B180" s="173"/>
       <c r="C180" s="105">
         <v>44256</v>
@@ -24359,7 +24359,7 @@
       </c>
       <c r="AV180" s="84"/>
     </row>
-    <row r="181" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:48">
       <c r="B181" s="173" t="s">
         <v>50</v>
       </c>
@@ -24491,7 +24491,7 @@
       </c>
       <c r="AV181" s="84"/>
     </row>
-    <row r="182" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:48">
       <c r="B182" s="173"/>
       <c r="C182" s="104">
         <v>44317</v>
@@ -24621,7 +24621,7 @@
       </c>
       <c r="AV182" s="84"/>
     </row>
-    <row r="183" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:48">
       <c r="B183" s="173"/>
       <c r="C183" s="104">
         <v>44348</v>
@@ -24751,7 +24751,7 @@
       </c>
       <c r="AV183" s="84"/>
     </row>
-    <row r="184" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:48">
       <c r="B184" s="173"/>
       <c r="C184" s="104">
         <v>44378</v>
@@ -24881,7 +24881,7 @@
       </c>
       <c r="AV184" s="84"/>
     </row>
-    <row r="185" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:48">
       <c r="B185" s="173"/>
       <c r="C185" s="104">
         <v>44409</v>
@@ -25011,7 +25011,7 @@
       </c>
       <c r="AV185" s="84"/>
     </row>
-    <row r="186" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:48">
       <c r="B186" s="173"/>
       <c r="C186" s="104">
         <v>44440</v>
@@ -25141,7 +25141,7 @@
       </c>
       <c r="AV186" s="84"/>
     </row>
-    <row r="187" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:48">
       <c r="B187" s="173"/>
       <c r="C187" s="104">
         <v>44470</v>
@@ -25271,7 +25271,7 @@
       </c>
       <c r="AV187" s="84"/>
     </row>
-    <row r="188" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:48">
       <c r="B188" s="173"/>
       <c r="C188" s="104">
         <v>44501</v>
@@ -25401,7 +25401,7 @@
       </c>
       <c r="AV188" s="84"/>
     </row>
-    <row r="189" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:48">
       <c r="B189" s="173"/>
       <c r="C189" s="85">
         <v>44531</v>
@@ -25531,7 +25531,7 @@
       </c>
       <c r="AV189" s="84"/>
     </row>
-    <row r="190" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:48">
       <c r="B190" s="173"/>
       <c r="C190" s="85">
         <v>44562</v>
@@ -25661,7 +25661,7 @@
       </c>
       <c r="AV190" s="84"/>
     </row>
-    <row r="191" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:48">
       <c r="B191" s="173"/>
       <c r="C191" s="85">
         <v>44593</v>
@@ -25791,7 +25791,7 @@
       </c>
       <c r="AV191" s="84"/>
     </row>
-    <row r="192" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:48">
       <c r="B192" s="173"/>
       <c r="C192" s="90">
         <v>44621</v>
@@ -25921,7 +25921,7 @@
       </c>
       <c r="AV192" s="84"/>
     </row>
-    <row r="193" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:48">
       <c r="B193" s="173" t="s">
         <v>51</v>
       </c>
@@ -26053,7 +26053,7 @@
       </c>
       <c r="AV193" s="84"/>
     </row>
-    <row r="194" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:48">
       <c r="B194" s="173"/>
       <c r="C194" s="104">
         <v>44682</v>
@@ -26183,7 +26183,7 @@
       </c>
       <c r="AV194" s="84"/>
     </row>
-    <row r="195" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:48">
       <c r="B195" s="173"/>
       <c r="C195" s="104">
         <v>44713</v>
@@ -26313,7 +26313,7 @@
       </c>
       <c r="AV195" s="84"/>
     </row>
-    <row r="196" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:48">
       <c r="B196" s="173"/>
       <c r="C196" s="104">
         <v>44743</v>
@@ -26443,7 +26443,7 @@
       </c>
       <c r="AV196" s="84"/>
     </row>
-    <row r="197" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:48">
       <c r="B197" s="173"/>
       <c r="C197" s="104">
         <v>44774</v>
@@ -26573,7 +26573,7 @@
       </c>
       <c r="AV197" s="84"/>
     </row>
-    <row r="198" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:48">
       <c r="B198" s="173"/>
       <c r="C198" s="104">
         <v>44805</v>
@@ -26703,7 +26703,7 @@
       </c>
       <c r="AV198" s="84"/>
     </row>
-    <row r="199" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:48">
       <c r="B199" s="173"/>
       <c r="C199" s="104">
         <v>44835</v>
@@ -26833,7 +26833,7 @@
       </c>
       <c r="AV199" s="84"/>
     </row>
-    <row r="200" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:48">
       <c r="B200" s="173"/>
       <c r="C200" s="104">
         <v>44866</v>
@@ -26962,7 +26962,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="201" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:48">
       <c r="B201" s="173"/>
       <c r="C201" s="85">
         <v>44896</v>
@@ -27091,7 +27091,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="202" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:48">
       <c r="B202" s="173"/>
       <c r="C202" s="85">
         <v>44927</v>
@@ -27220,7 +27220,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="203" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:48">
       <c r="B203" s="173"/>
       <c r="C203" s="85">
         <v>44958</v>
@@ -27349,7 +27349,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="204" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:48">
       <c r="B204" s="173"/>
       <c r="C204" s="90">
         <v>44986</v>
@@ -27478,7 +27478,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="205" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:48">
       <c r="B205" s="173" t="s">
         <v>52</v>
       </c>
@@ -27610,7 +27610,7 @@
       </c>
       <c r="AV205" s="84"/>
     </row>
-    <row r="206" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:48">
       <c r="B206" s="173"/>
       <c r="C206" s="104">
         <v>45047</v>
@@ -27740,7 +27740,7 @@
       </c>
       <c r="AV206" s="84"/>
     </row>
-    <row r="207" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:48">
       <c r="B207" s="173"/>
       <c r="C207" s="104">
         <v>45078</v>
@@ -27870,7 +27870,7 @@
       </c>
       <c r="AV207" s="84"/>
     </row>
-    <row r="208" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:48">
       <c r="B208" s="173"/>
       <c r="C208" s="104">
         <v>45108</v>
@@ -28000,7 +28000,7 @@
       </c>
       <c r="AV208" s="84"/>
     </row>
-    <row r="209" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:48">
       <c r="B209" s="173"/>
       <c r="C209" s="104">
         <v>45139</v>
@@ -28130,7 +28130,7 @@
       </c>
       <c r="AV209" s="84"/>
     </row>
-    <row r="210" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:48">
       <c r="B210" s="173"/>
       <c r="C210" s="104">
         <v>45170</v>
@@ -28260,7 +28260,7 @@
       </c>
       <c r="AV210" s="84"/>
     </row>
-    <row r="211" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:48">
       <c r="B211" s="173"/>
       <c r="C211" s="104">
         <v>45200</v>
@@ -28390,7 +28390,7 @@
       </c>
       <c r="AV211" s="84"/>
     </row>
-    <row r="212" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:48">
       <c r="B212" s="173"/>
       <c r="C212" s="104">
         <v>45231</v>
@@ -28519,7 +28519,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="213" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:48">
       <c r="B213" s="173"/>
       <c r="C213" s="155">
         <v>45261</v>
@@ -28648,7 +28648,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="214" spans="2:48" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="2:48" ht="13" thickBot="1">
       <c r="B214" s="174"/>
       <c r="C214" s="144">
         <v>45292</v>
@@ -28777,7 +28777,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="215" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:48">
       <c r="B215" s="173"/>
       <c r="C215" s="163" t="s">
         <v>53</v>
@@ -28906,7 +28906,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="216" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:48">
       <c r="B216" s="173"/>
       <c r="C216" s="90">
         <v>45352</v>
@@ -29035,7 +29035,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="217" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:48">
       <c r="B217" s="173" t="s">
         <v>55</v>
       </c>
@@ -29167,7 +29167,7 @@
       </c>
       <c r="AV217" s="84"/>
     </row>
-    <row r="218" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:48">
       <c r="B218" s="173"/>
       <c r="C218" s="104">
         <v>45413</v>
@@ -29297,7 +29297,7 @@
       </c>
       <c r="AV218" s="84"/>
     </row>
-    <row r="219" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:48">
       <c r="B219" s="173"/>
       <c r="C219" s="104">
         <v>45444</v>
@@ -29427,7 +29427,7 @@
       </c>
       <c r="AV219" s="84"/>
     </row>
-    <row r="220" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:48">
       <c r="B220" s="173"/>
       <c r="C220" s="104">
         <v>45474</v>
@@ -29557,7 +29557,7 @@
       </c>
       <c r="AV220" s="84"/>
     </row>
-    <row r="221" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:48">
       <c r="B221" s="173"/>
       <c r="C221" s="104">
         <v>45505</v>
@@ -29687,7 +29687,7 @@
       </c>
       <c r="AV221" s="84"/>
     </row>
-    <row r="222" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:48">
       <c r="B222" s="173"/>
       <c r="C222" s="104">
         <v>45536</v>
@@ -29817,7 +29817,7 @@
       </c>
       <c r="AV222" s="84"/>
     </row>
-    <row r="223" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:48">
       <c r="B223" s="173"/>
       <c r="C223" s="104">
         <v>45566</v>
@@ -29947,7 +29947,7 @@
       </c>
       <c r="AV223" s="84"/>
     </row>
-    <row r="224" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:48">
       <c r="B224" s="173"/>
       <c r="C224" s="104">
         <v>45597</v>
@@ -30076,7 +30076,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="225" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:48">
       <c r="B225" s="173"/>
       <c r="C225" s="155">
         <v>45627</v>
@@ -30205,7 +30205,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="226" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:48">
       <c r="B226" s="174"/>
       <c r="C226" s="104">
         <v>45658</v>
@@ -30334,7 +30334,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="227" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:48">
       <c r="B227" s="173"/>
       <c r="C227" s="104">
         <v>45689</v>
@@ -30463,7 +30463,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="228" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:48">
       <c r="B228" s="173"/>
       <c r="C228" s="90">
         <v>45717</v>
@@ -30592,7 +30592,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="229" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:48">
       <c r="B229" s="173" t="s">
         <v>73</v>
       </c>
@@ -30724,7 +30724,7 @@
       </c>
       <c r="AV229" s="84"/>
     </row>
-    <row r="230" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:48">
       <c r="B230" s="173"/>
       <c r="C230" s="104">
         <v>45778</v>
@@ -30854,7 +30854,7 @@
       </c>
       <c r="AV230" s="84"/>
     </row>
-    <row r="231" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:48">
       <c r="B231" s="173"/>
       <c r="C231" s="104">
         <v>45809</v>
@@ -30984,7 +30984,7 @@
       </c>
       <c r="AV231" s="84"/>
     </row>
-    <row r="232" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:48">
       <c r="B232" s="173"/>
       <c r="C232" s="104">
         <v>45839</v>
@@ -31114,7 +31114,7 @@
       </c>
       <c r="AV232" s="84"/>
     </row>
-    <row r="233" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:48">
       <c r="B233" s="173"/>
       <c r="C233" s="104">
         <v>45870</v>
@@ -31244,7 +31244,7 @@
       </c>
       <c r="AV233" s="84"/>
     </row>
-    <row r="234" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:48">
       <c r="B234" s="173"/>
       <c r="C234" s="104">
         <v>45901</v>
@@ -31374,7 +31374,7 @@
       </c>
       <c r="AV234" s="84"/>
     </row>
-    <row r="235" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:48">
       <c r="B235" s="173"/>
       <c r="C235" s="104">
         <v>45931</v>
@@ -31504,47 +31504,119 @@
       </c>
       <c r="AV235" s="84"/>
     </row>
-    <row r="236" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:48">
       <c r="B236" s="173"/>
       <c r="C236" s="104">
         <v>45962</v>
       </c>
-      <c r="D236" s="51"/>
-      <c r="E236" s="51"/>
-      <c r="F236" s="3"/>
-      <c r="G236" s="87"/>
-      <c r="H236" s="11"/>
-      <c r="I236" s="11"/>
-      <c r="J236" s="3"/>
-      <c r="K236" s="87"/>
-      <c r="L236" s="3"/>
-      <c r="M236" s="3"/>
-      <c r="N236" s="88"/>
-      <c r="O236" s="88"/>
-      <c r="P236" s="3"/>
-      <c r="Q236" s="3"/>
-      <c r="R236" s="3"/>
-      <c r="S236" s="3"/>
-      <c r="T236" s="3"/>
-      <c r="U236" s="3"/>
-      <c r="V236" s="53"/>
-      <c r="W236" s="53"/>
-      <c r="X236" s="54"/>
-      <c r="Y236" s="53"/>
-      <c r="Z236" s="2"/>
-      <c r="AA236" s="2"/>
-      <c r="AB236" s="18"/>
-      <c r="AC236" s="3"/>
-      <c r="AD236" s="18"/>
-      <c r="AE236" s="18"/>
-      <c r="AF236" s="9"/>
-      <c r="AG236" s="9"/>
-      <c r="AH236" s="3"/>
-      <c r="AI236" s="3"/>
-      <c r="AJ236" s="3"/>
-      <c r="AK236" s="3"/>
-      <c r="AL236" s="3"/>
-      <c r="AM236" s="3"/>
+      <c r="D236" s="51">
+        <v>12.8972515877183</v>
+      </c>
+      <c r="E236" s="51">
+        <v>40.3595505187794</v>
+      </c>
+      <c r="F236" s="3">
+        <v>4412862</v>
+      </c>
+      <c r="G236" s="87">
+        <v>4514602</v>
+      </c>
+      <c r="H236" s="11">
+        <v>0.61640673780313204</v>
+      </c>
+      <c r="I236" s="11">
+        <v>0.61768319512793124</v>
+      </c>
+      <c r="J236" s="3">
+        <v>2746148</v>
+      </c>
+      <c r="K236" s="87">
+        <v>2794326</v>
+      </c>
+      <c r="L236" s="3">
+        <v>154121</v>
+      </c>
+      <c r="M236" s="3">
+        <v>156483</v>
+      </c>
+      <c r="N236" s="88">
+        <v>2.1528256001877355E-2</v>
+      </c>
+      <c r="O236" s="88">
+        <v>2.1409842866149456E-2</v>
+      </c>
+      <c r="P236" s="3">
+        <v>9394</v>
+      </c>
+      <c r="Q236" s="3">
+        <v>9521</v>
+      </c>
+      <c r="R236" s="3">
+        <v>1485</v>
+      </c>
+      <c r="S236" s="3">
+        <v>1500</v>
+      </c>
+      <c r="T236" s="3">
+        <v>177</v>
+      </c>
+      <c r="U236" s="3">
+        <v>177</v>
+      </c>
+      <c r="V236" s="53">
+        <v>7159010</v>
+      </c>
+      <c r="W236" s="53">
+        <v>7308928</v>
+      </c>
+      <c r="X236" s="54">
+        <v>0.84440825860176605</v>
+      </c>
+      <c r="Y236" s="53">
+        <v>6171719.1647256883</v>
+      </c>
+      <c r="Z236" s="2">
+        <v>11.9868109303428</v>
+      </c>
+      <c r="AA236" s="2">
+        <v>59.695553737043099</v>
+      </c>
+      <c r="AB236" s="18">
+        <v>178823</v>
+      </c>
+      <c r="AC236" s="3">
+        <v>29602</v>
+      </c>
+      <c r="AD236" s="18">
+        <v>295278</v>
+      </c>
+      <c r="AE236" s="18">
+        <v>301760.56728778465</v>
+      </c>
+      <c r="AF236" s="9">
+        <v>9.1727835271524594</v>
+      </c>
+      <c r="AG236" s="9">
+        <v>53.604371276766997</v>
+      </c>
+      <c r="AH236" s="3">
+        <v>797416</v>
+      </c>
+      <c r="AI236" s="3">
+        <v>71428</v>
+      </c>
+      <c r="AJ236" s="3">
+        <v>1207449</v>
+      </c>
+      <c r="AK236" s="3">
+        <v>1234782.5403726709</v>
+      </c>
+      <c r="AL236" s="3">
+        <v>1669006</v>
+      </c>
+      <c r="AM236" s="3">
+        <v>1710325.420289855</v>
+      </c>
       <c r="AO236" s="44" t="s">
         <v>35</v>
       </c>
@@ -31561,7 +31633,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="237" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:48">
       <c r="B237" s="173"/>
       <c r="C237" s="155">
         <v>45992</v>
@@ -31618,7 +31690,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="238" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:48">
       <c r="B238" s="174"/>
       <c r="C238" s="104">
         <v>46023</v>
@@ -31675,7 +31747,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="239" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:48">
       <c r="B239" s="173"/>
       <c r="C239" s="104">
         <v>46054</v>
@@ -31732,7 +31804,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="240" spans="2:48" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:48">
       <c r="B240" s="173"/>
       <c r="C240" s="90">
         <v>46082</v>
@@ -31789,7 +31861,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="241" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:39" s="166" customFormat="1">
       <c r="B241" s="165" t="s">
         <v>54</v>
       </c>
@@ -31830,7 +31902,7 @@
       <c r="AL241" s="167"/>
       <c r="AM241" s="167"/>
     </row>
-    <row r="242" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:39" s="166" customFormat="1">
       <c r="B242" s="170" t="s">
         <v>62</v>
       </c>
@@ -31842,7 +31914,7 @@
       <c r="Y242" s="172"/>
       <c r="AF242" s="171"/>
     </row>
-    <row r="243" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:39" s="166" customFormat="1">
       <c r="B243" s="170" t="s">
         <v>63</v>
       </c>
@@ -31852,7 +31924,7 @@
       <c r="S243" s="168"/>
       <c r="AF243" s="171"/>
     </row>
-    <row r="244" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:39" s="166" customFormat="1">
       <c r="B244" s="170" t="s">
         <v>64</v>
       </c>
@@ -31862,7 +31934,7 @@
       <c r="S244" s="168"/>
       <c r="AF244" s="171"/>
     </row>
-    <row r="245" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:39" s="166" customFormat="1">
       <c r="B245" s="170" t="s">
         <v>65</v>
       </c>
@@ -31872,7 +31944,7 @@
       <c r="S245" s="168"/>
       <c r="AF245" s="171"/>
     </row>
-    <row r="246" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:39" s="166" customFormat="1">
       <c r="B246" s="170" t="s">
         <v>66</v>
       </c>
@@ -31882,7 +31954,7 @@
       <c r="S246" s="168"/>
       <c r="AF246" s="171"/>
     </row>
-    <row r="247" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:39" s="166" customFormat="1">
       <c r="B247" s="170" t="s">
         <v>67</v>
       </c>
@@ -31891,7 +31963,7 @@
       <c r="R247" s="168"/>
       <c r="S247" s="168"/>
     </row>
-    <row r="248" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:39" s="166" customFormat="1">
       <c r="B248" s="170" t="s">
         <v>68</v>
       </c>
@@ -31900,7 +31972,7 @@
       <c r="R248" s="168"/>
       <c r="S248" s="168"/>
     </row>
-    <row r="249" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:39" s="166" customFormat="1">
       <c r="B249" s="170" t="s">
         <v>69</v>
       </c>
@@ -31909,7 +31981,7 @@
       <c r="R249" s="168"/>
       <c r="S249" s="168"/>
     </row>
-    <row r="250" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:39" s="166" customFormat="1">
       <c r="B250" s="170" t="s">
         <v>70</v>
       </c>
@@ -31918,7 +31990,7 @@
       <c r="R250" s="168"/>
       <c r="S250" s="168"/>
     </row>
-    <row r="251" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:39" s="166" customFormat="1">
       <c r="B251" s="170" t="s">
         <v>71</v>
       </c>
@@ -31927,7 +31999,7 @@
       <c r="R251" s="168"/>
       <c r="S251" s="168"/>
     </row>
-    <row r="252" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:39" s="166" customFormat="1">
       <c r="B252" s="170" t="s">
         <v>56</v>
       </c>
@@ -31936,7 +32008,7 @@
       <c r="R252" s="168"/>
       <c r="S252" s="168"/>
     </row>
-    <row r="253" spans="2:39" s="166" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:39" s="166" customFormat="1">
       <c r="P253" s="168"/>
       <c r="Q253" s="168"/>
       <c r="R253" s="168"/>
@@ -31944,11 +32016,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B205:B216"/>
-    <mergeCell ref="B193:B204"/>
-    <mergeCell ref="B181:B192"/>
-    <mergeCell ref="B133:B144"/>
-    <mergeCell ref="B121:B132"/>
     <mergeCell ref="B217:B228"/>
     <mergeCell ref="B229:B240"/>
     <mergeCell ref="AL11:AM11"/>
@@ -31965,6 +32032,11 @@
     <mergeCell ref="B169:B180"/>
     <mergeCell ref="B145:B156"/>
     <mergeCell ref="B157:B168"/>
+    <mergeCell ref="B205:B216"/>
+    <mergeCell ref="B193:B204"/>
+    <mergeCell ref="B181:B192"/>
+    <mergeCell ref="B133:B144"/>
+    <mergeCell ref="B121:B132"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.15748031496062992" right="0.15748031496062992" top="0.15748031496062992" bottom="0.35433070866141736" header="0.35433070866141736" footer="0.15748031496062992"/>
@@ -31980,12 +32052,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5fcde14c-a1ff-41f1-a210-ce352d4e962b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -32235,21 +32310,28 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5fcde14c-a1ff-41f1-a210-ce352d4e962b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D406A7D-7898-42E9-9873-AA8507271B14}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{768FE709-DAC2-484B-B042-CA0F22E8B0F4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="5fcde14c-a1ff-41f1-a210-ce352d4e962b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="58b241f0-c181-42d5-839a-5e9ae10f42c8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -32275,19 +32357,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{768FE709-DAC2-484B-B042-CA0F22E8B0F4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D406A7D-7898-42E9-9873-AA8507271B14}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="5fcde14c-a1ff-41f1-a210-ce352d4e962b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="58b241f0-c181-42d5-839a-5e9ae10f42c8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Latest unemployment and NHS data
</commit_message>
<xml_diff>
--- a/downloads/latest-waiting-list.xlsx
+++ b/downloads/latest-waiting-list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs.sharepoint.com/sites/X24_PAT-UECandAP/Shared Documents/UEC and AP/RTT/Monthly RTT Report/25_26/202511 Nov/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs.sharepoint.com/sites/X24_PAT-UECandAP/Shared Documents/UEC and AP/RTT/Monthly RTT Report/25_26/202512 Dec/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="8_{3DAF2501-AF2A-431F-A0A7-AB4BE36DDE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47A27414-C726-47FC-9079-B059AFC63892}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{3DAF2501-AF2A-431F-A0A7-AB4BE36DDE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{242CB25B-8F91-4F1C-AF33-53C36A53D465}"/>
   <bookViews>
     <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -667,7 +667,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>April 2007 to November 2025</t>
+      <t>April 2007 to December 2025</t>
     </r>
   </si>
 </sst>
@@ -1574,7 +1574,7 @@
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -30600,46 +30600,46 @@
         <v>45748</v>
       </c>
       <c r="D229" s="52">
-        <v>13.2586792742547</v>
+        <v>13.2581646249944</v>
       </c>
       <c r="E229" s="52">
-        <v>42.262696453345697</v>
+        <v>42.261807186054803</v>
       </c>
       <c r="F229" s="83">
-        <v>4413743</v>
+        <v>4413682</v>
       </c>
       <c r="G229" s="98">
-        <v>4413743</v>
+        <v>4413682</v>
       </c>
       <c r="H229" s="22">
-        <v>0.59731778682903902</v>
+        <v>0.59732618403004978</v>
       </c>
       <c r="I229" s="138">
-        <v>0.59731778682903902</v>
+        <v>0.59732618403004978</v>
       </c>
       <c r="J229" s="3">
-        <v>2975528</v>
+        <v>2975383</v>
       </c>
       <c r="K229" s="131">
-        <v>2975528</v>
+        <v>2975383</v>
       </c>
       <c r="L229" s="83">
-        <v>190068</v>
+        <v>190023</v>
       </c>
       <c r="M229" s="83">
-        <v>190068</v>
+        <v>190023</v>
       </c>
       <c r="N229" s="99">
-        <v>2.5722158518749684E-2</v>
+        <v>2.5716785547291843E-2</v>
       </c>
       <c r="O229" s="99">
-        <v>2.5722158518749684E-2</v>
+        <v>2.5716785547291843E-2</v>
       </c>
       <c r="P229" s="83">
-        <v>9258</v>
+        <v>9244</v>
       </c>
       <c r="Q229" s="83">
-        <v>9258</v>
+        <v>9244</v>
       </c>
       <c r="R229" s="83">
         <v>1361</v>
@@ -30654,58 +30654,58 @@
         <v>171</v>
       </c>
       <c r="V229" s="101">
-        <v>7389271</v>
+        <v>7389065</v>
       </c>
       <c r="W229" s="101">
-        <v>7389271</v>
+        <v>7389065</v>
       </c>
       <c r="X229" s="56">
         <v>0.84363713381192296</v>
       </c>
       <c r="Y229" s="101">
-        <v>6233863.4073995622</v>
+        <v>6233689.6181499967</v>
       </c>
       <c r="Z229" s="24">
-        <v>10.631983805668</v>
+        <v>10.6356458361452</v>
       </c>
       <c r="AA229" s="24">
-        <v>59.334945930563499</v>
+        <v>59.335486624928897</v>
       </c>
       <c r="AB229" s="23">
-        <v>189402</v>
+        <v>189364</v>
       </c>
       <c r="AC229" s="3">
-        <v>27931</v>
+        <v>27930</v>
       </c>
       <c r="AD229" s="23">
-        <v>305987</v>
+        <v>305948</v>
       </c>
       <c r="AE229" s="23">
-        <v>305987</v>
+        <v>305948</v>
       </c>
       <c r="AF229" s="25">
-        <v>8.1415339865278593</v>
+        <v>8.1485113781953498</v>
       </c>
       <c r="AG229" s="25">
-        <v>52.456803054032903</v>
+        <v>52.453944792482403</v>
       </c>
       <c r="AH229" s="83">
-        <v>780158</v>
+        <v>780447</v>
       </c>
       <c r="AI229" s="83">
         <v>59497</v>
       </c>
       <c r="AJ229" s="83">
-        <v>1143854</v>
+        <v>1144146</v>
       </c>
       <c r="AK229" s="83">
-        <v>1143854</v>
+        <v>1144146</v>
       </c>
       <c r="AL229" s="83">
-        <v>1712674</v>
+        <v>1707444</v>
       </c>
       <c r="AM229" s="83">
-        <v>1712674</v>
+        <v>1707444</v>
       </c>
       <c r="AO229" s="43" t="s">
         <v>35</v>
@@ -30730,46 +30730,46 @@
         <v>45778</v>
       </c>
       <c r="D230" s="51">
-        <v>13.5683561806774</v>
+        <v>13.5697948901055</v>
       </c>
       <c r="E230" s="51">
-        <v>42.523734390788</v>
+        <v>42.526729349836899</v>
       </c>
       <c r="F230" s="3">
-        <v>4484636</v>
+        <v>4482076</v>
       </c>
       <c r="G230" s="87">
-        <v>4484636</v>
+        <v>4482076</v>
       </c>
       <c r="H230" s="11">
-        <v>0.60937050111169888</v>
+        <v>0.60931300511830555</v>
       </c>
       <c r="I230" s="11">
-        <v>0.60937050111169888</v>
+        <v>0.60931300511830555</v>
       </c>
       <c r="J230" s="3">
-        <v>2874821</v>
+        <v>2873874</v>
       </c>
       <c r="K230" s="87">
-        <v>2874821</v>
+        <v>2873874</v>
       </c>
       <c r="L230" s="3">
-        <v>196920</v>
+        <v>196839</v>
       </c>
       <c r="M230" s="3">
-        <v>196920</v>
+        <v>196839</v>
       </c>
       <c r="N230" s="88">
-        <v>2.6757408868616259E-2</v>
+        <v>2.6759154154120134E-2</v>
       </c>
       <c r="O230" s="88">
-        <v>2.6757408868616259E-2</v>
+        <v>2.6759154154120134E-2</v>
       </c>
       <c r="P230" s="3">
-        <v>11522</v>
+        <v>11473</v>
       </c>
       <c r="Q230" s="3">
-        <v>11522</v>
+        <v>11473</v>
       </c>
       <c r="R230" s="3">
         <v>1237</v>
@@ -30778,64 +30778,64 @@
         <v>1237</v>
       </c>
       <c r="T230" s="3">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U230" s="3">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="V230" s="53">
-        <v>7359457</v>
+        <v>7355950</v>
       </c>
       <c r="W230" s="53">
-        <v>7359457</v>
+        <v>7355950</v>
       </c>
       <c r="X230" s="54">
         <v>0.84603034683079004</v>
       </c>
       <c r="Y230" s="101">
-        <v>6226323.9581962852</v>
+        <v>6223356.92976995</v>
       </c>
       <c r="Z230" s="2">
-        <v>10.9674869310213</v>
+        <v>10.9749394209922</v>
       </c>
       <c r="AA230" s="2">
-        <v>59.2</v>
+        <v>59.2041910331384</v>
       </c>
       <c r="AB230" s="18">
-        <v>197240</v>
+        <v>197111</v>
       </c>
       <c r="AC230" s="3">
-        <v>28842</v>
+        <v>28840</v>
       </c>
       <c r="AD230" s="18">
-        <v>313121</v>
+        <v>312800</v>
       </c>
       <c r="AE230" s="18">
-        <v>313121</v>
+        <v>312800</v>
       </c>
       <c r="AF230" s="9">
-        <v>8.6684623340803295</v>
+        <v>8.6649054982817901</v>
       </c>
       <c r="AG230" s="9">
-        <v>53.358956014838398</v>
+        <v>53.349929341105799</v>
       </c>
       <c r="AH230" s="3">
-        <v>813696</v>
+        <v>814674</v>
       </c>
       <c r="AI230" s="3">
-        <v>67356</v>
+        <v>67364</v>
       </c>
       <c r="AJ230" s="3">
-        <v>1187052</v>
+        <v>1187895</v>
       </c>
       <c r="AK230" s="3">
-        <v>1187052</v>
+        <v>1187895</v>
       </c>
       <c r="AL230" s="3">
-        <v>1752664</v>
+        <v>1757217</v>
       </c>
       <c r="AM230" s="3">
-        <v>1752664</v>
+        <v>1757217</v>
       </c>
       <c r="AO230" s="44" t="s">
         <v>35</v>
@@ -30860,46 +30860,46 @@
         <v>45809</v>
       </c>
       <c r="D231" s="51">
-        <v>13.3955249109422</v>
+        <v>13.397750439012601</v>
       </c>
       <c r="E231" s="51">
-        <v>41.805975856585199</v>
+        <v>41.806544140236703</v>
       </c>
       <c r="F231" s="3">
-        <v>4534245</v>
+        <v>4533070</v>
       </c>
       <c r="G231" s="87">
-        <v>4534245</v>
+        <v>4533070</v>
       </c>
       <c r="H231" s="11">
-        <v>0.61529936414811492</v>
+        <v>0.61525120808877942</v>
       </c>
       <c r="I231" s="11">
-        <v>0.61529936414811492</v>
+        <v>0.61525120808877942</v>
       </c>
       <c r="J231" s="3">
-        <v>2834924</v>
+        <v>2834766</v>
       </c>
       <c r="K231" s="87">
-        <v>2834924</v>
+        <v>2834766</v>
       </c>
       <c r="L231" s="3">
-        <v>191813</v>
+        <v>191755</v>
       </c>
       <c r="M231" s="3">
-        <v>191813</v>
+        <v>191755</v>
       </c>
       <c r="N231" s="88">
-        <v>2.6029122143894381E-2</v>
+        <v>2.6025959318312732E-2</v>
       </c>
       <c r="O231" s="88">
-        <v>2.6029122143894381E-2</v>
+        <v>2.6025959318312732E-2</v>
       </c>
       <c r="P231" s="3">
-        <v>10517</v>
+        <v>10486</v>
       </c>
       <c r="Q231" s="3">
-        <v>10517</v>
+        <v>10486</v>
       </c>
       <c r="R231" s="3">
         <v>1103</v>
@@ -30914,58 +30914,58 @@
         <v>182</v>
       </c>
       <c r="V231" s="53">
-        <v>7369169</v>
+        <v>7367836</v>
       </c>
       <c r="W231" s="53">
-        <v>7369169</v>
+        <v>7367836</v>
       </c>
       <c r="X231" s="54">
         <v>0.84576100373929897</v>
       </c>
       <c r="Y231" s="101">
-        <v>6232555.7701645261</v>
+        <v>6231428.3707465418</v>
       </c>
       <c r="Z231" s="2">
-        <v>11.359585838343399</v>
+        <v>11.365281859471001</v>
       </c>
       <c r="AA231" s="2">
-        <v>59.325013789299497</v>
+        <v>59.327440706012098</v>
       </c>
       <c r="AB231" s="18">
-        <v>200081</v>
+        <v>199995</v>
       </c>
       <c r="AC231" s="3">
         <v>30411</v>
       </c>
       <c r="AD231" s="18">
-        <v>320947</v>
+        <v>320661</v>
       </c>
       <c r="AE231" s="18">
-        <v>320947</v>
+        <v>320661</v>
       </c>
       <c r="AF231" s="9">
-        <v>8.8358184177960197</v>
+        <v>8.8220349223611905</v>
       </c>
       <c r="AG231" s="9">
-        <v>53.7005202114958</v>
+        <v>53.690363295241298</v>
       </c>
       <c r="AH231" s="3">
-        <v>842493</v>
+        <v>843632</v>
       </c>
       <c r="AI231" s="3">
-        <v>72603</v>
+        <v>72601</v>
       </c>
       <c r="AJ231" s="3">
-        <v>1237188</v>
+        <v>1237971</v>
       </c>
       <c r="AK231" s="3">
-        <v>1237188</v>
+        <v>1237971</v>
       </c>
       <c r="AL231" s="3">
-        <v>1828833</v>
+        <v>1828309</v>
       </c>
       <c r="AM231" s="3">
-        <v>1828833</v>
+        <v>1828309</v>
       </c>
       <c r="AO231" s="44" t="s">
         <v>35</v>
@@ -30990,52 +30990,52 @@
         <v>45839</v>
       </c>
       <c r="D232" s="121">
-        <v>13.0959121949747</v>
+        <v>13.0989688179403</v>
       </c>
       <c r="E232" s="121">
-        <v>41.795638080698701</v>
+        <v>41.796676193350301</v>
       </c>
       <c r="F232" s="122">
-        <v>4469950</v>
+        <v>4468469</v>
       </c>
       <c r="G232" s="128">
-        <v>4530213</v>
+        <v>4528732</v>
       </c>
       <c r="H232" s="11">
-        <v>0.61226287218328534</v>
+        <v>0.61220097539081597</v>
       </c>
       <c r="I232" s="11">
-        <v>0.61285680658445119</v>
+        <v>0.61279580919746057</v>
       </c>
       <c r="J232" s="3">
-        <v>2830754</v>
+        <v>2830554</v>
       </c>
       <c r="K232" s="87">
-        <v>2861747</v>
+        <v>2861547</v>
       </c>
       <c r="L232" s="3">
-        <v>189480</v>
+        <v>189416</v>
       </c>
       <c r="M232" s="3">
-        <v>191277</v>
+        <v>191213</v>
       </c>
       <c r="N232" s="88">
-        <v>2.5953661455114466E-2</v>
+        <v>2.5950870411012541E-2</v>
       </c>
       <c r="O232" s="88">
-        <v>2.5876357556047381E-2</v>
+        <v>2.587358339245379E-2</v>
       </c>
       <c r="P232" s="3">
-        <v>11902</v>
+        <v>11863</v>
       </c>
       <c r="Q232" s="3">
-        <v>11942</v>
+        <v>11903</v>
       </c>
       <c r="R232" s="3">
-        <v>1429</v>
+        <v>1417</v>
       </c>
       <c r="S232" s="3">
-        <v>1431</v>
+        <v>1419</v>
       </c>
       <c r="T232" s="3">
         <v>244</v>
@@ -31044,58 +31044,58 @@
         <v>244</v>
       </c>
       <c r="V232" s="53">
-        <v>7300704</v>
+        <v>7299023</v>
       </c>
       <c r="W232" s="53">
-        <v>7391960</v>
+        <v>7390279</v>
       </c>
       <c r="X232" s="54">
         <v>0.84407551027574101</v>
       </c>
       <c r="Y232" s="101">
-        <v>6239372.4089378668</v>
+        <v>6237953.5180050926</v>
       </c>
       <c r="Z232" s="127">
-        <v>10.989213364904</v>
+        <v>10.9936200999737</v>
       </c>
       <c r="AA232" s="2">
-        <v>59.092716319824703</v>
+        <v>59.094222343921103</v>
       </c>
       <c r="AB232" s="3">
-        <v>205547</v>
+        <v>205490</v>
       </c>
       <c r="AC232" s="3">
         <v>30621</v>
       </c>
       <c r="AD232" s="3">
-        <v>328738</v>
+        <v>328683</v>
       </c>
       <c r="AE232" s="3">
-        <v>333417.95238095237</v>
+        <v>333362.95238095237</v>
       </c>
       <c r="AF232" s="121">
-        <v>8.17374579026826</v>
+        <v>8.1680844268958293</v>
       </c>
       <c r="AG232" s="26">
-        <v>53.2444435431538</v>
+        <v>53.240549967553498</v>
       </c>
       <c r="AH232" s="123">
-        <v>889923</v>
+        <v>890339</v>
       </c>
       <c r="AI232" s="3">
-        <v>73109</v>
+        <v>73106</v>
       </c>
       <c r="AJ232" s="122">
-        <v>1297445</v>
+        <v>1297865</v>
       </c>
       <c r="AK232" s="122">
-        <v>1315161.5714285714</v>
+        <v>1315581.5714285714</v>
       </c>
       <c r="AL232" s="122">
-        <v>1914582</v>
+        <v>1913956</v>
       </c>
       <c r="AM232" s="122">
-        <v>1943163.3333333333</v>
+        <v>1942537.3333333333</v>
       </c>
       <c r="AO232" s="44" t="s">
         <v>35</v>
@@ -31120,52 +31120,52 @@
         <v>45870</v>
       </c>
       <c r="D233" s="51">
-        <v>13.447446693921499</v>
+        <v>13.4515398550725</v>
       </c>
       <c r="E233" s="51">
-        <v>42.155670406132003</v>
+        <v>42.157048613049099</v>
       </c>
       <c r="F233" s="3">
-        <v>4459975</v>
+        <v>4458454</v>
       </c>
       <c r="G233" s="87">
-        <v>4520238</v>
+        <v>4518717</v>
       </c>
       <c r="H233" s="11">
-        <v>0.60978335889151158</v>
+        <v>0.6097151178088156</v>
       </c>
       <c r="I233" s="11">
-        <v>0.61040677958777567</v>
+        <v>0.61033952076364884</v>
       </c>
       <c r="J233" s="3">
-        <v>2854057</v>
+        <v>2853902</v>
       </c>
       <c r="K233" s="87">
-        <v>2885050</v>
+        <v>2884895</v>
       </c>
       <c r="L233" s="3">
-        <v>188752</v>
+        <v>188702</v>
       </c>
       <c r="M233" s="3">
-        <v>190549</v>
+        <v>190499</v>
       </c>
       <c r="N233" s="88">
-        <v>2.5806832674508395E-2</v>
+        <v>2.5805909887319491E-2</v>
       </c>
       <c r="O233" s="88">
-        <v>2.5731477290282294E-2</v>
+        <v>2.5730548818603677E-2</v>
       </c>
       <c r="P233" s="3">
-        <v>12753</v>
+        <v>12715</v>
       </c>
       <c r="Q233" s="3">
-        <v>12793</v>
+        <v>12755</v>
       </c>
       <c r="R233" s="3">
-        <v>1416</v>
+        <v>1397</v>
       </c>
       <c r="S233" s="3">
-        <v>1418</v>
+        <v>1399</v>
       </c>
       <c r="T233" s="3">
         <v>168</v>
@@ -31174,58 +31174,58 @@
         <v>168</v>
       </c>
       <c r="V233" s="53">
-        <v>7314032</v>
+        <v>7312356</v>
       </c>
       <c r="W233" s="53">
-        <v>7405288</v>
+        <v>7403612</v>
       </c>
       <c r="X233" s="54">
         <v>0.84411356832520701</v>
       </c>
       <c r="Y233" s="101">
-        <v>6250904.0781558352</v>
+        <v>6249489.343815323</v>
       </c>
       <c r="Z233" s="2">
-        <v>10.898190045248899</v>
+        <v>10.902131075755401</v>
       </c>
       <c r="AA233" s="2">
-        <v>59.355073859987101</v>
+        <v>59.3573859987155</v>
       </c>
       <c r="AB233" s="18">
-        <v>179596</v>
+        <v>179524</v>
       </c>
       <c r="AC233" s="3">
         <v>26991</v>
       </c>
       <c r="AD233" s="18">
-        <v>287654</v>
+        <v>287582</v>
       </c>
       <c r="AE233" s="18">
-        <v>291723.52380952379</v>
+        <v>291651.52380952379</v>
       </c>
       <c r="AF233" s="9">
-        <v>8.1701091961583998</v>
+        <v>8.1631099565960792</v>
       </c>
       <c r="AG233" s="9">
-        <v>53.456230031948898</v>
+        <v>53.451347843450499</v>
       </c>
       <c r="AH233" s="3">
-        <v>753114</v>
+        <v>753595</v>
       </c>
       <c r="AI233" s="3">
         <v>62250</v>
       </c>
       <c r="AJ233" s="3">
-        <v>1096542</v>
+        <v>1097031</v>
       </c>
       <c r="AK233" s="3">
-        <v>1111947.7142857143</v>
+        <v>1112436.7142857143</v>
       </c>
       <c r="AL233" s="3">
-        <v>1602458</v>
+        <v>1602010</v>
       </c>
       <c r="AM233" s="3">
-        <v>1627311.3333333333</v>
+        <v>1626863.3333333333</v>
       </c>
       <c r="AO233" s="44" t="s">
         <v>35</v>
@@ -31250,28 +31250,28 @@
         <v>45901</v>
       </c>
       <c r="D234" s="51">
-        <v>13.354927205562801</v>
+        <v>13.357978200639099</v>
       </c>
       <c r="E234" s="51">
-        <v>41.812171800816998</v>
+        <v>41.814069930069898</v>
       </c>
       <c r="F234" s="3">
-        <v>4506959</v>
+        <v>4505684</v>
       </c>
       <c r="G234" s="87">
-        <v>4567222</v>
+        <v>4565947</v>
       </c>
       <c r="H234" s="11">
-        <v>0.61754501494686287</v>
+        <v>0.61747979585283763</v>
       </c>
       <c r="I234" s="11">
-        <v>0.61807391977988058</v>
+        <v>0.61800959888599971</v>
       </c>
       <c r="J234" s="3">
-        <v>2791228</v>
+        <v>2791209</v>
       </c>
       <c r="K234" s="87">
-        <v>2822221</v>
+        <v>2822202</v>
       </c>
       <c r="L234" s="3">
         <v>178532</v>
@@ -31280,10 +31280,10 @@
         <v>180329</v>
       </c>
       <c r="N234" s="88">
-        <v>2.4462513772256042E-2</v>
+        <v>2.4466851850506784E-2</v>
       </c>
       <c r="O234" s="88">
-        <v>2.4403598485027898E-2</v>
+        <v>2.4407872662015884E-2</v>
       </c>
       <c r="P234" s="3">
         <v>12782</v>
@@ -31304,58 +31304,58 @@
         <v>150</v>
       </c>
       <c r="V234" s="53">
-        <v>7298187</v>
+        <v>7296893</v>
       </c>
       <c r="W234" s="53">
-        <v>7389443</v>
+        <v>7388149</v>
       </c>
       <c r="X234" s="54">
         <v>0.84410501656553005</v>
       </c>
       <c r="Y234" s="53">
-        <v>6237465.9059250401</v>
+        <v>6236373.6340336045</v>
       </c>
       <c r="Z234" s="2">
-        <v>11.887499999999999</v>
+        <v>11.8813335097235</v>
       </c>
       <c r="AA234" s="2">
-        <v>60.038077367205602</v>
+        <v>60.035508083140897</v>
       </c>
       <c r="AB234" s="18">
-        <v>194802</v>
+        <v>194892</v>
       </c>
       <c r="AC234" s="3">
         <v>31282</v>
       </c>
       <c r="AD234" s="18">
-        <v>318971</v>
+        <v>319060</v>
       </c>
       <c r="AE234" s="18">
-        <v>323447.47619047621</v>
+        <v>323536.47619047621</v>
       </c>
       <c r="AF234" s="9">
-        <v>9.3058858949269894</v>
+        <v>9.3003522398843899</v>
       </c>
       <c r="AG234" s="9">
-        <v>53.3881096475614</v>
+        <v>53.384469562121701</v>
       </c>
       <c r="AH234" s="3">
-        <v>856494</v>
+        <v>856897</v>
       </c>
       <c r="AI234" s="3">
         <v>72606</v>
       </c>
       <c r="AJ234" s="3">
-        <v>1276491</v>
+        <v>1276900</v>
       </c>
       <c r="AK234" s="3">
-        <v>1293437.2857142857</v>
+        <v>1293846.2857142857</v>
       </c>
       <c r="AL234" s="3">
-        <v>1818704</v>
+        <v>1818303</v>
       </c>
       <c r="AM234" s="3">
-        <v>1846042.6666666667</v>
+        <v>1845641.6666666667</v>
       </c>
       <c r="AO234" s="44" t="s">
         <v>35</v>
@@ -31638,42 +31638,114 @@
       <c r="C237" s="155">
         <v>45992</v>
       </c>
-      <c r="D237" s="156"/>
-      <c r="E237" s="156"/>
-      <c r="F237" s="92"/>
-      <c r="G237" s="93"/>
-      <c r="H237" s="157"/>
-      <c r="I237" s="157"/>
-      <c r="J237" s="92"/>
-      <c r="K237" s="93"/>
-      <c r="L237" s="92"/>
-      <c r="M237" s="92"/>
-      <c r="N237" s="158"/>
-      <c r="O237" s="158"/>
-      <c r="P237" s="92"/>
-      <c r="Q237" s="92"/>
-      <c r="R237" s="92"/>
-      <c r="S237" s="92"/>
-      <c r="T237" s="92"/>
-      <c r="U237" s="92"/>
-      <c r="V237" s="159"/>
-      <c r="W237" s="159"/>
-      <c r="X237" s="55"/>
-      <c r="Y237" s="159"/>
-      <c r="Z237" s="160"/>
-      <c r="AA237" s="160"/>
-      <c r="AB237" s="161"/>
-      <c r="AC237" s="92"/>
-      <c r="AD237" s="161"/>
-      <c r="AE237" s="92"/>
-      <c r="AF237" s="162"/>
-      <c r="AG237" s="162"/>
-      <c r="AH237" s="92"/>
-      <c r="AI237" s="92"/>
-      <c r="AJ237" s="92"/>
-      <c r="AK237" s="92"/>
-      <c r="AL237" s="92"/>
-      <c r="AM237" s="92"/>
+      <c r="D237" s="156">
+        <v>13.445756276791199</v>
+      </c>
+      <c r="E237" s="156">
+        <v>40.778064850126803</v>
+      </c>
+      <c r="F237" s="92">
+        <v>4424207</v>
+      </c>
+      <c r="G237" s="93">
+        <v>4484470</v>
+      </c>
+      <c r="H237" s="157">
+        <v>0.61450528527600889</v>
+      </c>
+      <c r="I237" s="157">
+        <v>0.61507938685042129</v>
+      </c>
+      <c r="J237" s="92">
+        <v>2775417</v>
+      </c>
+      <c r="K237" s="93">
+        <v>2806410</v>
+      </c>
+      <c r="L237" s="92">
+        <v>138711</v>
+      </c>
+      <c r="M237" s="92">
+        <v>140508</v>
+      </c>
+      <c r="N237" s="158">
+        <v>1.9266422802079665E-2</v>
+      </c>
+      <c r="O237" s="158">
+        <v>1.927174771769663E-2</v>
+      </c>
+      <c r="P237" s="92">
+        <v>7304</v>
+      </c>
+      <c r="Q237" s="92">
+        <v>7344</v>
+      </c>
+      <c r="R237" s="92">
+        <v>1512</v>
+      </c>
+      <c r="S237" s="92">
+        <v>1514</v>
+      </c>
+      <c r="T237" s="92">
+        <v>223</v>
+      </c>
+      <c r="U237" s="92">
+        <v>223</v>
+      </c>
+      <c r="V237" s="159">
+        <v>7199624</v>
+      </c>
+      <c r="W237" s="159">
+        <v>7290880</v>
+      </c>
+      <c r="X237" s="55">
+        <v>0.84649182564120296</v>
+      </c>
+      <c r="Y237" s="159">
+        <v>6171670.3217309341</v>
+      </c>
+      <c r="Z237" s="160">
+        <v>11.5610972568579</v>
+      </c>
+      <c r="AA237" s="160">
+        <v>59.641484184914802</v>
+      </c>
+      <c r="AB237" s="161">
+        <v>165977</v>
+      </c>
+      <c r="AC237" s="92">
+        <v>26749</v>
+      </c>
+      <c r="AD237" s="161">
+        <v>270395</v>
+      </c>
+      <c r="AE237" s="92">
+        <v>274668</v>
+      </c>
+      <c r="AF237" s="162">
+        <v>8.6158325360430208</v>
+      </c>
+      <c r="AG237" s="162">
+        <v>52.397246053534602</v>
+      </c>
+      <c r="AH237" s="92">
+        <v>764866</v>
+      </c>
+      <c r="AI237" s="92">
+        <v>59091</v>
+      </c>
+      <c r="AJ237" s="92">
+        <v>1136006</v>
+      </c>
+      <c r="AK237" s="92">
+        <v>1152182</v>
+      </c>
+      <c r="AL237" s="92">
+        <v>1617349</v>
+      </c>
+      <c r="AM237" s="92">
+        <v>1643445</v>
+      </c>
       <c r="AO237" s="44" t="s">
         <v>35</v>
       </c>
@@ -32052,6 +32124,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -32063,9 +32144,9 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBC83FE296745C42B8674DB72D139957" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1620ab93aeaa7a1859ac03483cce22a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="58b241f0-c181-42d5-839a-5e9ae10f42c8" xmlns:ns3="5fcde14c-a1ff-41f1-a210-ce352d4e962b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e3ffe406c8d8d2ef81f68edbb59c5bc" ns1:_="" ns2:_="" ns3:_="">
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBC83FE296745C42B8674DB72D139957" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2def9819561c10c3a5c0a4c5418f01f5">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="58b241f0-c181-42d5-839a-5e9ae10f42c8" xmlns:ns3="5fcde14c-a1ff-41f1-a210-ce352d4e962b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cae15ef64808bdcf281a127d0c686fcb" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="58b241f0-c181-42d5-839a-5e9ae10f42c8"/>
     <xsd:import namespace="5fcde14c-a1ff-41f1-a210-ce352d4e962b"/>
@@ -32309,16 +32390,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D406A7D-7898-42E9-9873-AA8507271B14}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{768FE709-DAC2-484B-B042-CA0F22E8B0F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -32336,8 +32416,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D871FA2-06AF-494D-8248-499F53A1A506}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFD97FDE-CF18-486F-9CED-C5BD0110329A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -32356,14 +32436,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D406A7D-7898-42E9-9873-AA8507271B14}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{37c354b2-85b0-47f5-b222-07b48d774ee3}" enabled="0" method="" siteId="{37c354b2-85b0-47f5-b222-07b48d774ee3}" removed="1"/>

</xml_diff>